<commit_message>
[FEAT]: add new features
- Add two new model but in this case is only RNA
- improve wording in some files for better claritty
- fix the schendule for the gantt_chart
- add the appendices directory
</commit_message>
<xml_diff>
--- a/Thesis/02_Chapters/gantt_chart.xlsx
+++ b/Thesis/02_Chapters/gantt_chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Dropbox/LuisAngelGH/Incremental Learning/Incremental-Learning/Thesis/02_Chapters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{857EEEFE-49FE-3D40-91B4-E61CC2DDDBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7822A0B-82A4-CB4E-8067-FC232B87AB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7100" yWindow="1040" windowWidth="28040" windowHeight="17440" xr2:uid="{A1AB2931-02A3-5944-88AC-D60CF2DBCCC7}"/>
+    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{A1AB2931-02A3-5944-88AC-D60CF2DBCCC7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
   <si>
     <t>Actividad</t>
   </si>
@@ -90,6 +90,42 @@
   </si>
   <si>
     <t>Examen profesional</t>
+  </si>
+  <si>
+    <t>Oct-nov 2025</t>
+  </si>
+  <si>
+    <t>Dic-ene 2026</t>
+  </si>
+  <si>
+    <t>Feb-mar 2026</t>
+  </si>
+  <si>
+    <t>Abr-may 2026</t>
+  </si>
+  <si>
+    <t>Jun-jul 2026</t>
+  </si>
+  <si>
+    <t>Ago-sep 2026</t>
+  </si>
+  <si>
+    <t>Oct-nov 2026</t>
+  </si>
+  <si>
+    <t>Dic-ene 2027</t>
+  </si>
+  <si>
+    <t>Feb-mar 2027</t>
+  </si>
+  <si>
+    <t>Abr-may 2027</t>
+  </si>
+  <si>
+    <t>Jun-jul 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planteamiento de la Investigación </t>
   </si>
 </sst>
 </file>
@@ -97,9 +133,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode=";;;"/>
+    <numFmt numFmtId="164" formatCode=";;;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -116,6 +152,18 @@
     </font>
     <font>
       <sz val="16"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="15"/>
       <color theme="1"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
@@ -162,15 +210,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -507,10 +573,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C9DBB7-2AF8-9F43-943C-F33C424B8108}">
-  <dimension ref="C2:J12"/>
+  <dimension ref="C2:O27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="45.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="77.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -518,6 +584,10 @@
     <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:10" ht="20" x14ac:dyDescent="0.2">
@@ -806,22 +876,586 @@
         <v>1</v>
       </c>
     </row>
+    <row r="17" spans="3:15" ht="19" x14ac:dyDescent="0.2">
+      <c r="C17" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C18" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+    </row>
+    <row r="20" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C20" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="2">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+    </row>
+    <row r="21" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="2">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2">
+        <v>1</v>
+      </c>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+    </row>
+    <row r="22" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="2">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2">
+        <v>1</v>
+      </c>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+    </row>
+    <row r="23" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>1</v>
+      </c>
+      <c r="J23" s="2">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2">
+        <v>1</v>
+      </c>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+    </row>
+    <row r="24" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="2">
+        <v>1</v>
+      </c>
+      <c r="K24" s="2">
+        <v>1</v>
+      </c>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C25" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="2">
+        <v>1</v>
+      </c>
+      <c r="M25" s="2">
+        <v>1</v>
+      </c>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C26" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="2">
+        <v>1</v>
+      </c>
+      <c r="N26" s="2">
+        <v>1</v>
+      </c>
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="3:15" ht="20" x14ac:dyDescent="0.2">
+      <c r="C27" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="C2:J2">
+    <cfRule type="dataBar" priority="26">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BBA953A6-AE92-DD41-B79D-BB51CF940AB8}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:J12">
+    <cfRule type="dataBar" priority="23">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{C422AF66-3E4C-4443-BC55-6DD880FB1B5D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18:E18">
+    <cfRule type="dataBar" priority="22">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="dataBar" priority="21">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{6ADDBDD4-CC87-CC42-8F4B-7EA0ED2D82D3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E20">
+    <cfRule type="dataBar" priority="20">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{622FC78C-9FD3-D14F-9CD5-5876317FA14E}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F20">
+    <cfRule type="dataBar" priority="19">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F8A7C9AC-7071-2A42-95F8-E198A9568A68}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F21">
+    <cfRule type="dataBar" priority="18">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F3808704-EC62-E14D-919D-6323487222BB}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G21">
+    <cfRule type="dataBar" priority="17">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{33DC49CD-9EBD-A948-93AC-9DD2C034BB3A}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="dataBar" priority="16">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9F9CDC62-D3FA-9647-9D10-02F43CF65536}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22">
+    <cfRule type="dataBar" priority="15">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{CBBF0FFB-C6C4-4E49-B3D0-F639BF5637A5}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H22">
+    <cfRule type="dataBar" priority="14">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F12D7536-955E-9846-AA78-10A58D728B8D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
+    <cfRule type="dataBar" priority="13">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{AF5BBB01-7FE2-B148-B20A-FB09026DC4A6}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23">
+    <cfRule type="dataBar" priority="12">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{035712E5-968C-FC47-886A-2C9605FFB98F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I22">
+    <cfRule type="dataBar" priority="11">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{AB4B5E83-73B0-7E41-9C50-03859B831E5F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J23">
+    <cfRule type="dataBar" priority="10">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2B28EDCA-91C7-A24C-805E-2C1BDDFE2EA3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{D8811C63-F5DA-EF46-818B-2319EC1A1582}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J24">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{714893BE-B2C9-2E47-B766-939C6F21DCBD}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K24">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A5C8CF39-526B-2844-9F66-CC04E969CE73}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L23">
+    <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{1F10EB31-0458-234D-8862-A4D24F826AA9}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L25">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{EF3F07DD-141E-0143-9D4E-CF3569CF4237}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M25">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BBA953A6-AE92-DD41-B79D-BB51CF940AB8}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:J12">
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A22619C1-D8F1-0148-9446-AF449B7171AC}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M26">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{1FFC7F0A-751D-AE4B-992F-7C42A6E496E4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N26">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BCCBA02A-77F9-7948-AB69-B69B541844BD}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O27">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -830,7 +1464,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C422AF66-3E4C-4443-BC55-6DD880FB1B5D}</x14:id>
+          <x14:id>{E41A1CBE-21EA-1F41-9A02-C571B0FA6A0A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -864,6 +1498,292 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D3:J12</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D18:E18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{6ADDBDD4-CC87-CC42-8F4B-7EA0ED2D82D3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E19</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{622FC78C-9FD3-D14F-9CD5-5876317FA14E}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F8A7C9AC-7071-2A42-95F8-E198A9568A68}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>F20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F3808704-EC62-E14D-919D-6323487222BB}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>F21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{33DC49CD-9EBD-A948-93AC-9DD2C034BB3A}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9F9CDC62-D3FA-9647-9D10-02F43CF65536}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{CBBF0FFB-C6C4-4E49-B3D0-F639BF5637A5}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F12D7536-955E-9846-AA78-10A58D728B8D}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{AF5BBB01-7FE2-B148-B20A-FB09026DC4A6}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{035712E5-968C-FC47-886A-2C9605FFB98F}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{AB4B5E83-73B0-7E41-9C50-03859B831E5F}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2B28EDCA-91C7-A24C-805E-2C1BDDFE2EA3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>J23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{D8811C63-F5DA-EF46-818B-2319EC1A1582}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>K23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{714893BE-B2C9-2E47-B766-939C6F21DCBD}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>J24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A5C8CF39-526B-2844-9F66-CC04E969CE73}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>K24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{1F10EB31-0458-234D-8862-A4D24F826AA9}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>L23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{EF3F07DD-141E-0143-9D4E-CF3569CF4237}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>L25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A22619C1-D8F1-0148-9446-AF449B7171AC}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>M25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{1FFC7F0A-751D-AE4B-992F-7C42A6E496E4}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>M26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{BCCBA02A-77F9-7948-AB69-B69B541844BD}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>N26</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{E41A1CBE-21EA-1F41-9A02-C571B0FA6A0A}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O27</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
[FEAT]: add the section of result in the document
</commit_message>
<xml_diff>
--- a/Thesis/02_Chapters/gantt_chart.xlsx
+++ b/Thesis/02_Chapters/gantt_chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Dropbox/LuisAngelGH/Incremental Learning/Incremental-Learning/Thesis/02_Chapters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/Library/CloudStorage/Dropbox/LuisAngelGH/Incremental Learning/Incremental-Learning/Thesis/02_Chapters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7822A0B-82A4-CB4E-8067-FC232B87AB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A752198-5312-3841-B898-04CAF28EAD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{A1AB2931-02A3-5944-88AC-D60CF2DBCCC7}"/>
+    <workbookView xWindow="-38400" yWindow="-6340" windowWidth="38400" windowHeight="24000" xr2:uid="{A1AB2931-02A3-5944-88AC-D60CF2DBCCC7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="36">
   <si>
     <t>Actividad</t>
   </si>
@@ -126,6 +126,24 @@
   </si>
   <si>
     <t xml:space="preserve">Planteamiento de la Investigación </t>
+  </si>
+  <si>
+    <t>Ago</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dic</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -135,7 +153,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=";;;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -168,8 +186,27 @@
       <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -180,6 +217,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
+        <bgColor rgb="FFFFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B084"/>
+        <bgColor rgb="FFF4B084"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF4B084"/>
       </patternFill>
     </fill>
   </fills>
@@ -210,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -227,7 +288,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -238,6 +299,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -257,7 +339,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -573,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C9DBB7-2AF8-9F43-943C-F33C424B8108}">
-  <dimension ref="C2:O27"/>
+  <dimension ref="C2:O38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="77.5" bestFit="1" customWidth="1"/>
@@ -1132,6 +1214,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="33" spans="3:8" ht="21" x14ac:dyDescent="0.2">
+      <c r="C33" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="3:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="C34" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+    </row>
+    <row r="35" spans="3:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="C35" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="16"/>
+      <c r="E35" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" spans="3:8" ht="22" x14ac:dyDescent="0.2">
+      <c r="C36" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="16"/>
+    </row>
+    <row r="37" spans="3:8" ht="22" x14ac:dyDescent="0.2">
+      <c r="C37" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="3:8" ht="22" x14ac:dyDescent="0.2">
+      <c r="C38" s="14"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="16"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="C2:J2">
     <cfRule type="dataBar" priority="26">
@@ -1147,6 +1309,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D18:E18">
+    <cfRule type="dataBar" priority="22">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D3:J12">
     <cfRule type="dataBar" priority="23">
       <dataBar>
@@ -1161,20 +1337,6 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D18:E18">
-    <cfRule type="dataBar" priority="22">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E19">
     <cfRule type="dataBar" priority="21">
       <dataBar>
@@ -1231,6 +1393,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="dataBar" priority="16">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9F9CDC62-D3FA-9647-9D10-02F43CF65536}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G21">
     <cfRule type="dataBar" priority="17">
       <dataBar>
@@ -1245,20 +1421,6 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G20">
-    <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9F9CDC62-D3FA-9647-9D10-02F43CF65536}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="G22">
     <cfRule type="dataBar" priority="15">
       <dataBar>
@@ -1301,6 +1463,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I22">
+    <cfRule type="dataBar" priority="11">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{AB4B5E83-73B0-7E41-9C50-03859B831E5F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I23">
     <cfRule type="dataBar" priority="12">
       <dataBar>
@@ -1315,20 +1491,6 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I22">
-    <cfRule type="dataBar" priority="11">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AB4B5E83-73B0-7E41-9C50-03859B831E5F}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J23">
     <cfRule type="dataBar" priority="10">
       <dataBar>
@@ -1343,6 +1505,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J24">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{714893BE-B2C9-2E47-B766-939C6F21DCBD}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K23">
     <cfRule type="dataBar" priority="9">
       <dataBar>
@@ -1357,20 +1533,6 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J24">
-    <cfRule type="dataBar" priority="8">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB628"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{714893BE-B2C9-2E47-B766-939C6F21DCBD}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K24">
     <cfRule type="dataBar" priority="7">
       <dataBar>
@@ -1470,6 +1632,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -1487,6 +1650,19 @@
           <xm:sqref>C2:J2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D18:E18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C422AF66-3E4C-4443-BC55-6DD880FB1B5D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1500,19 +1676,6 @@
           <xm:sqref>D3:J12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28F7E483-7E98-BB40-BBAD-E97CCF24D9E8}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D18:E18</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{6ADDBDD4-CC87-CC42-8F4B-7EA0ED2D82D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1565,6 +1728,19 @@
           <xm:sqref>F21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9F9CDC62-D3FA-9647-9D10-02F43CF65536}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G20</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{33DC49CD-9EBD-A948-93AC-9DD2C034BB3A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1578,19 +1754,6 @@
           <xm:sqref>G21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9F9CDC62-D3FA-9647-9D10-02F43CF65536}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>G20</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{CBBF0FFB-C6C4-4E49-B3D0-F639BF5637A5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1630,6 +1793,19 @@
           <xm:sqref>H23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{AB4B5E83-73B0-7E41-9C50-03859B831E5F}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I22</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{035712E5-968C-FC47-886A-2C9605FFB98F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1643,19 +1819,6 @@
           <xm:sqref>I23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AB4B5E83-73B0-7E41-9C50-03859B831E5F}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I22</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{2B28EDCA-91C7-A24C-805E-2C1BDDFE2EA3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1669,6 +1832,19 @@
           <xm:sqref>J23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{714893BE-B2C9-2E47-B766-939C6F21DCBD}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFFB628"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>J24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{D8811C63-F5DA-EF46-818B-2319EC1A1582}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -1680,19 +1856,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>K23</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{714893BE-B2C9-2E47-B766-939C6F21DCBD}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFFB628"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>J24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{A5C8CF39-526B-2844-9F66-CC04E969CE73}">

</xml_diff>